<commit_message>
Update Finding Informaion field
</commit_message>
<xml_diff>
--- a/Coverage_Matrix_17_Kategori_Serangan.validated.xlsx
+++ b/Coverage_Matrix_17_Kategori_Serangan.validated.xlsx
@@ -643,26 +643,26 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.531719+00:00</t>
+          <t>2026-09-29T16:35:28.157462+00:00</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>01-49dac1cfcb1343ac9a6d6bb73441440d</t>
+          <t>01-88decaa979044d96b27c22047330332b</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>12a65994-9305-489c-aa68-1e8f5ca4e8bc</t>
+          <t>77f4f6b3-452d-4f29-a4c6-2fecabccd057</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>8ff2fd74-d74b-46f0-b3f8-b019462be59a</t>
+          <t>73d4e001-e330-4435-876c-ca20a4dd090f</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>0.022</v>
+        <v>0.032</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -746,26 +746,26 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.576045+00:00</t>
+          <t>2026-09-29T16:35:28.275417+00:00</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>02-e4a6206d99f744ffb5458540bc02d046</t>
+          <t>02-e12ac6281bcb47a7a38239a39aebdffc</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>e0fba84b-3626-4eb8-8108-a63d9f9fc4ad</t>
+          <t>fc664d9b-c89e-4ee2-8582-db5e8dce4577</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>d74f1e35-a63c-47aa-93fd-9c5db737e141</t>
+          <t>381ffd99-598e-4c35-9e0d-0534f7cb672c</t>
         </is>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>0.023</v>
+        <v>0.024</v>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
@@ -784,7 +784,7 @@
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -849,26 +849,26 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.633494+00:00</t>
+          <t>2026-09-29T16:35:28.340305+00:00</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>03-7bc91ae8a2824bc49347c0c560d06459</t>
+          <t>03-849648bab9e840e98eab7de7ee7cb006</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>59db5617-9e45-4ba6-8115-f733a7a102f3</t>
+          <t>5e095a7f-a665-480f-b064-9b741f639007</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2032db33-54a1-42ad-8bb2-180fbc317ebe</t>
+          <t>b069121d-fd1b-40a8-9c09-0cd51fd964b3</t>
         </is>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>0.022</v>
+        <v>0.033</v>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -952,26 +952,26 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.668820+00:00</t>
+          <t>2026-09-29T16:35:28.413561+00:00</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>04-92559cbc9c3341618e7a55894b7da1af</t>
+          <t>04-bdb875b42073403d860191277d5a16ce</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>6fc66207-c440-45d0-a60a-f9eadbbbd726</t>
+          <t>c71af8e1-efdd-485c-8d85-1a474669a38a</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>f035d8e6-5869-42aa-a944-6eaf53f5c89e</t>
+          <t>732e584b-d2c2-4953-af5e-37e0b5a6a76f</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>0.019</v>
+        <v>0.023</v>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1055,26 +1055,26 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.697327+00:00</t>
+          <t>2026-09-29T16:35:28.623721+00:00</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>05-3ec6deac30944f65bb1bc020a74003e2</t>
+          <t>05-469ced4968a64612b2831daa428f0ea0</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>9448b081-3bf5-497e-9d6c-6c7c50c8d535</t>
+          <t>a44cf170-2ca3-436f-b5b4-21c242ae83c6</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>ae222b19-d13b-4377-8028-cb79f7de0795</t>
+          <t>acdc2ca9-03a3-4001-886b-9954396dbde5</t>
         </is>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>0.019</v>
+        <v>0.057</v>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1158,26 +1158,26 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.726358+00:00</t>
+          <t>2026-09-29T16:35:28.859024+00:00</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>06-d80049518b3f4968b31aab0ffc910c46</t>
+          <t>06-a028b9aa752e4ead8094210b05650a45</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>be39cdc0-6b8f-442c-a0a7-8817c9ef44e2</t>
+          <t>52a9d781-d410-4183-b802-d5533f40812f</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>abd51fcd-742b-4712-9268-e0c7fe17cc3f</t>
+          <t>cfbc04c1-03c9-4313-8d31-ee0ee0a50640</t>
         </is>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>0.019</v>
+        <v>0.021</v>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1261,26 +1261,26 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.754632+00:00</t>
+          <t>2026-09-29T16:35:28.916115+00:00</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>07-e6196c543a284e1e8e03ac5c9937b589</t>
+          <t>07-6abd62604d074101bbb29698726db280</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>f5920149-5955-4a1e-a42c-bcd8be2cda29</t>
+          <t>0b4b619e-176c-422d-be40-8c99e9c41e0a</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>57fa3ed6-a126-4ae9-96c3-f755a75ac35f</t>
+          <t>320d2cb4-822b-428f-ac06-b8199d4b9e08</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>0.02</v>
+        <v>0.021</v>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1364,26 +1364,26 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.784056+00:00</t>
+          <t>2026-09-29T16:35:28.992072+00:00</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>08-bc2352a0a6c5474f8d805c24d0b935f4</t>
+          <t>08-c590777712da446089c6f46a689898a0</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>99077ef9-0676-4a5e-8dc9-0b353d986e61</t>
+          <t>cb9c6a1c-1b49-42f2-a88e-8a13efc14b77</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>7732cf44-d0d5-4b03-870d-b75ae3c8f8e4</t>
+          <t>5bbd3ffb-f8e0-41c6-b0a5-f0a320548889</t>
         </is>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>0.021</v>
+        <v>0.026</v>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1467,26 +1467,26 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.814611+00:00</t>
+          <t>2026-09-29T16:35:29.052953+00:00</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>09-ed1e374f5401409c9d47711b0befc400</t>
+          <t>09-f8b39ca776214ee9bd415d4912f2f838</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>887ae347-621a-4925-bb97-cb34a9c479bf</t>
+          <t>69d8cc64-6977-46ae-9120-cf64d54320bf</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>abfc4f03-fd6a-4f83-bc35-73a73af32c9d</t>
+          <t>e360876e-8646-4084-a6cf-ee25237f17f0</t>
         </is>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>0.032</v>
+        <v>0.024</v>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1570,26 +1570,26 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.855971+00:00</t>
+          <t>2026-09-29T16:35:29.215985+00:00</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>10-35357417e35c43ea9b906aaca5cc34a7</t>
+          <t>10-c4156cbeab8f4d398f201a14deeac54d</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>6bad9862-2400-4b61-b794-689d205034ac</t>
+          <t>57bcc18d-a91c-4eeb-856b-1a74b68ac188</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>728a32b5-3381-4e8a-a486-9c8c3f16c8bd</t>
+          <t>96365a34-8e35-48a0-ad2d-75a8cc2dc963</t>
         </is>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>0.02</v>
+        <v>0.022</v>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1673,26 +1673,26 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.885730+00:00</t>
+          <t>2026-09-29T16:35:29.285593+00:00</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>11-894a420dcd6f4ba594facfd3c2249540</t>
+          <t>11-b134b2f9a8024feeb92ff9edeaf66aab</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>fe086466-a000-4cce-8193-9129fe36192f</t>
+          <t>49eab17f-e6be-4063-a698-5446892f109e</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>9818f5a0-8ebf-4ac3-a91f-69ab69041e27</t>
+          <t>c25733ab-b7de-4067-8d01-176c5fbad345</t>
         </is>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>0.021</v>
+        <v>0.023</v>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1776,26 +1776,26 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.918472+00:00</t>
+          <t>2026-09-29T16:35:29.346078+00:00</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>12-34f5835451c446fcb56b7f17e138fbbc</t>
+          <t>12-7016c2fae6654b9f801dca1a9eff4fc0</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>1993808e-0cea-4034-88a2-8512a9558f35</t>
+          <t>2117f512-10af-484c-9aae-ff356ab31855</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>a4472d3c-cc6b-4e48-b979-90d1c27ba6f7</t>
+          <t>afd930c2-6fcd-4c25-8a7d-4fb33af4dfae</t>
         </is>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>0.03</v>
+        <v>0.023</v>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1879,26 +1879,26 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.958448+00:00</t>
+          <t>2026-09-29T16:35:29.407771+00:00</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>13-47612cce7d134f91a3cb06c7ba2df9a1</t>
+          <t>13-bf58b1c67b6a41ae90ea3141ad3c531f</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>e8f4a93a-9d74-49f2-a346-839c28800b44</t>
+          <t>95c20fd9-f67d-4b4e-a74d-b8e02b0f5f0c</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>326f1ff3-8887-4263-ba42-61ba50ffa492</t>
+          <t>23b6268f-c192-412f-b2ca-502292375302</t>
         </is>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>0.02</v>
+        <v>0.028</v>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -1982,26 +1982,26 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:22.988887+00:00</t>
+          <t>2026-09-29T16:35:29.474442+00:00</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>14-d4485fb4486c4710832e798af1919467</t>
+          <t>14-ba0f19289cc4417ea085981e2ec270c7</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>fcd2e312-c3a7-498d-99e4-7aae580c578b</t>
+          <t>e891b8a1-157e-4563-afe5-0e7527a71090</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>f8bd102c-2497-4f62-9eb1-94ceae39568f</t>
+          <t>647bc550-5e84-4c3c-98d8-263ff4826ce4</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>0.022</v>
+        <v>0.057</v>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -2085,12 +2085,12 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:23.021229+00:00</t>
+          <t>2026-09-29T16:35:29.651251+00:00</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>15-53ac4c8fe32d4e12bcd39b481ff31cb2</t>
+          <t>15-94c5d5b97c2549a08f58a4e1d078edb3</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -2190,26 +2190,26 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:23.021382+00:00</t>
+          <t>2026-09-29T16:35:29.651450+00:00</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>16-35aab881b38844a58c36ad3973688775</t>
+          <t>16-4ef6eb36339b4fd3aa759c2b12263958</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>ba983e66-5dbb-4a25-a264-dc2484dfb472</t>
+          <t>84895665-01fe-4236-8bcc-0d1b173c586d</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>55bedade-e4da-46c8-ab6e-f57164f10484</t>
+          <t>307a431d-5846-4dae-8740-41d3c115a13b</t>
         </is>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>0.021</v>
+        <v>0.022</v>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>
@@ -2293,26 +2293,26 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T13:34:23.052326+00:00</t>
+          <t>2026-09-29T16:35:29.719570+00:00</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>17-08e0bb31888f45c49f8276e8e4c64d94</t>
+          <t>17-59ea352af574484980780388c76fb691</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>6e7abb7b-a7bd-4b7c-9e92-bbbb7f0f8767</t>
+          <t>1deb8f4a-4e25-4be5-92f2-fceb7d34dde9</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>6eb22cff-ddd1-482d-a342-d0e5cd5235b6</t>
+          <t>11794828-0238-4a6b-b72c-7df42448864f</t>
         </is>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>0.019</v>
+        <v>0.022</v>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>Exact event UUID, expected category, and marker verified via dashboard_api</t>
+          <t>Exact event UUID, category, marker, and Attack Details fields verified via dashboard_api</t>
         </is>
       </c>
     </row>

</xml_diff>